<commit_message>
Fix UWP-D operating instructions source link
</commit_message>
<xml_diff>
--- a/quick-dial-cards-editable.xlsx
+++ b/quick-dial-cards-editable.xlsx
@@ -1794,7 +1794,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:E32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -2083,17 +2083,29 @@
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
+          <t>UWP-D operating instructions</t>
+        </is>
+      </c>
+      <c r="C31" s="11" t="inlineStr">
+        <is>
+          <t>https://pro.sony/support/res/manuals/5009/96c5bb8845154ae1e06fbe70a175ad9d/50099341M.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
           <t>UWP frequency lists</t>
         </is>
       </c>
-      <c r="C31" s="11" t="inlineStr">
+      <c r="C32" s="11" t="inlineStr">
         <is>
           <t>https://pro.sony/support/res/manuals/4530/63d2501a47358304ae6fe7185a0a2c9c/45307382M.pdf</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="12">
+  <mergeCells count="14">
     <mergeCell ref="B23:E23"/>
     <mergeCell ref="B8:E8"/>
     <mergeCell ref="A16:E16"/>
@@ -2101,14 +2113,17 @@
     <mergeCell ref="A28:E28"/>
     <mergeCell ref="B6:E6"/>
     <mergeCell ref="C31:E31"/>
+    <mergeCell ref="A32:B32"/>
     <mergeCell ref="B7:E7"/>
     <mergeCell ref="B24:E24"/>
     <mergeCell ref="B5:E5"/>
     <mergeCell ref="A31:B31"/>
     <mergeCell ref="A27:E27"/>
+    <mergeCell ref="C32:E32"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C31" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C32" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>